<commit_message>
feat: Add content on manage obligation home page
- adds content to details/summary
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/multi-year/xlsx/06-obligations-home-no-obligations.xlsx
+++ b/translations/welsh-translations/multi-year/xlsx/06-obligations-home-no-obligations.xlsx
@@ -76,7 +76,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="5" width="24" customWidth="1" hidden="1"/>
@@ -2247,8 +2247,386 @@
         </is>
       </c>
     </row>
+    <row r="56" ht="51" customHeight="1">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_heading</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">obligations_details_summary_heading</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prns-obligations-home-no-obligations</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/manage-your-recycling-obligations</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Why does the recycling obligations table already have tonnage awaiting acceptance?</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=1915-112595</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="51" customHeight="1">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_intro</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">obligations_details_summary_content_intro</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prns-obligations-home-no-obligations</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/manage-your-recycling-obligations</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tonnage awaiting acceptance is for PRNs or PERNs that have been issued to you but have not yet been accepted.</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=1915-112595</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="51" customHeight="1">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_before_list_1</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">obligations_details_summary_content_before_list_1</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prns-obligations-home-no-obligations</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/manage-your-recycling-obligations</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You have been issued at least one December waste PRN or PERN.</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=1915-112595</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="51" customHeight="1">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_before_list_2</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">obligations_details_summary_content_before_list_2</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prns-obligations-home-no-obligations</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/manage-your-recycling-obligations</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">These:</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=1915-112595</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="51" customHeight="1">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_bullet_1</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">obligations_details_summary_content_bullet_1</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prns-obligations-home-no-obligations</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/manage-your-recycling-obligations</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">are for packaging waste received for recycling at UK or overseas reprocessing sites in December</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=1915-112595</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="51" customHeight="1">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_bullet_2</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">obligations_details_summary_content_bullet_2</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prns-obligations-home-no-obligations</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/manage-your-recycling-obligations</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">can be accepted towards either your {0} or {1} recycling obligations</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=1915-112595</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="51" customHeight="1">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_bullet_3</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">obligations_details_summary_content_bullet_3</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prns-obligations-home-no-obligations</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/manage-your-recycling-obligations</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">have a blue tag to show which years you can accept them towards</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=1915-112595</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="51" customHeight="1">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_after_list</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">obligations_details_summary_content_after_list</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prns-obligations-home-no-obligations</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/manage-your-recycling-obligations</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A December waste PRN or PERN will appear under ‘Tonnage awaiting acceptance’ for both {0} and {1} until you accept it towards a specific year’s recycling obligations.</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=1915-112595</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="51" customHeight="1">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_end</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">obligations_details_summary_content_end</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prns-obligations-home-no-obligations</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/manage-your-recycling-obligations</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Once you accept the PRN or PERN towards a specific year, it is assigned to that year only and the blue tag is removed.</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=1915-112595</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:H55"/>
+  <autoFilter ref="A5:H64"/>
   <mergeCells count="3">
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="F2:H2"/>

</xml_diff>

<commit_message>
feat(Obligations page): Update multi-year content
- updates multi-year content  for new text before table on manage obligations page
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/multi-year/xlsx/06-obligations-home-no-obligations.xlsx
+++ b/translations/welsh-translations/multi-year/xlsx/06-obligations-home-no-obligations.xlsx
@@ -76,7 +76,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="5" width="24" customWidth="1" hidden="1"/>
@@ -150,17 +150,17 @@
     <row r="6" ht="51" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/PrnsObligation/ObligationsHome.en.resx::your_yyyy_recycling_obligations_will_be</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx::review_your_prns_and_perns</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/PrnsObligation/ObligationsHome.en.resx</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">your_yyyy_recycling_obligations_will_be</t>
+          <t xml:space="preserve">review_your_prns_and_perns</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -175,12 +175,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Your {0} recycling obligations will be calculated after:</t>
+          <t xml:space="preserve">Review your PRNs and PERNs</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Adolygu'ch PRNs a'ch PERNs</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -192,17 +192,17 @@
     <row r="7" ht="51" customHeight="1">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/PrnsObligation/ObligationsHome.en.resx::the_regulator_accepts_your_h1_and_h2_packaging_data_submissions</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx::review_your_prns_and_perns_yyyy</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/PrnsObligation/ObligationsHome.en.resx</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">the_regulator_accepts_your_h1_and_h2_packaging_data_submissions</t>
+          <t xml:space="preserve">review_your_prns_and_perns_yyyy</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -217,7 +217,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">the regulator accepts your H1 and H2 packaging data submissions</t>
+          <t xml:space="preserve">Review your PRNs and PERNs for {0}</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -234,7 +234,7 @@
     <row r="8" ht="51" customHeight="1">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx::review_your_prns_and_perns</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx::view_and_accept_prns_and_perns</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -244,7 +244,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">review_your_prns_and_perns</t>
+          <t xml:space="preserve">view_and_accept_prns_and_perns</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -259,12 +259,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Review your PRNs and PERNs</t>
+          <t xml:space="preserve">View and accept any issued PRNs and PERNs to meet your recycling obligations.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Adolygu'ch PRNs a'ch PERNs</t>
+          <t xml:space="preserve">Gweld a derbyn unrhyw PRNs a PERNs sydd wedi'u rhoi er mwyn cyflawni'ch rhwymedigaethau ailgylchu.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -276,7 +276,7 @@
     <row r="9" ht="51" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx::review_your_prns_and_perns_yyyy</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx::what_to_do_next</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -286,7 +286,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">review_your_prns_and_perns_yyyy</t>
+          <t xml:space="preserve">what_to_do_next</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -301,12 +301,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Review your PRNs and PERNs for {0}</t>
+          <t xml:space="preserve">What to do next</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Beth i'w wneud nesaf</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -318,7 +318,7 @@
     <row r="10" ht="51" customHeight="1">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx::view_and_accept_prns_and_perns</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx::accept_or_reject_prns_and_perns</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -328,7 +328,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">view_and_accept_prns_and_perns</t>
+          <t xml:space="preserve">accept_or_reject_prns_and_perns</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -343,12 +343,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">View and accept any issued PRNs and PERNs to meet your recycling obligations.</t>
+          <t xml:space="preserve">Accept or reject PRNs and PERNs</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gweld a derbyn unrhyw PRNs a PERNs sydd wedi'u rhoi er mwyn cyflawni'ch rhwymedigaethau ailgylchu.</t>
+          <t xml:space="preserve">Derbyn neu wrthod PRNs a PERNs</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -360,7 +360,7 @@
     <row r="11" ht="51" customHeight="1">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx::what_to_do_next</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx::accept_or_reject_prns_and_perns_yyyy</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -370,7 +370,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">what_to_do_next</t>
+          <t xml:space="preserve">accept_or_reject_prns_and_perns_yyyy</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -385,12 +385,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">What to do next</t>
+          <t xml:space="preserve">Accept or reject PRNs and PERNs for {0}</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beth i'w wneud nesaf</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -402,7 +402,7 @@
     <row r="12" ht="51" customHeight="1">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx::accept_or_reject_prns_and_perns</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx::search_prns_and_perns</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -412,7 +412,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">accept_or_reject_prns_and_perns</t>
+          <t xml:space="preserve">search_prns_and_perns</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -427,12 +427,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accept or reject PRNs and PERNs</t>
+          <t xml:space="preserve">Search PRNs and PERNs</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Derbyn neu wrthod PRNs a PERNs</t>
+          <t xml:space="preserve">Chwilio PRNs a PERNs</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -444,7 +444,7 @@
     <row r="13" ht="51" customHeight="1">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx::accept_or_reject_prns_and_perns_yyyy</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx::download_all_prns_and_perns</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -454,7 +454,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">accept_or_reject_prns_and_perns_yyyy</t>
+          <t xml:space="preserve">download_all_prns_and_perns</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -469,12 +469,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accept or reject PRNs and PERNs for {0}</t>
+          <t xml:space="preserve">Download a list of all PRNs and PERNs (CSV)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Lawrlwytho rhestr o'r holl PRNs a PERNs</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -486,7 +486,7 @@
     <row r="14" ht="51" customHeight="1">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx::search_prns_and_perns</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx::download_all_prns_and_perns_yyyy</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -496,7 +496,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">search_prns_and_perns</t>
+          <t xml:space="preserve">download_all_prns_and_perns_yyyy</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -511,12 +511,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Search PRNs and PERNs</t>
+          <t xml:space="preserve">Download a list of all PRNs and PERNs for {0} (CSV)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chwilio PRNs a PERNs</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -528,17 +528,17 @@
     <row r="15" ht="51" customHeight="1">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx::download_all_prns_and_perns</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsHeader.en.resx::compliance_scheme</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsHeader.en.resx</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">download_all_prns_and_perns</t>
+          <t xml:space="preserve">compliance_scheme</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -553,12 +553,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Download a list of all PRNs and PERNs (CSV)</t>
+          <t xml:space="preserve">Compliance Scheme</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lawrlwytho rhestr o'r holl PRNs a PERNs</t>
+          <t xml:space="preserve">Cynllun Cydymffurfio</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -570,17 +570,17 @@
     <row r="16" ht="51" customHeight="1">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx::download_all_prns_and_perns_yyyy</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsHeader.en.resx::january</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsHeader.en.resx</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">download_all_prns_and_perns_yyyy</t>
+          <t xml:space="preserve">january</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -595,12 +595,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Download a list of all PRNs and PERNs for {0} (CSV)</t>
+          <t xml:space="preserve">31 January</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">31 Ionawr </t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -612,7 +612,7 @@
     <row r="17" ht="51" customHeight="1">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsHeader.en.resx::compliance_scheme</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsHeader.en.resx::producer</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">compliance_scheme</t>
+          <t xml:space="preserve">producer</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -637,12 +637,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compliance Scheme</t>
+          <t xml:space="preserve">Producer</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cynllun Cydymffurfio</t>
+          <t xml:space="preserve">Cynhyrchydd</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -654,7 +654,7 @@
     <row r="18" ht="51" customHeight="1">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsHeader.en.resx::january</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsHeader.en.resx::regulator</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -664,7 +664,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">january</t>
+          <t xml:space="preserve">regulator</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -679,12 +679,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">31 January</t>
+          <t xml:space="preserve">Regulator</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t xml:space="preserve">31 Ionawr </t>
+          <t xml:space="preserve">Rheoleiddiwr</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -696,7 +696,7 @@
     <row r="19" ht="51" customHeight="1">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsHeader.en.resx::producer</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsHeader.en.resx::regulator_england</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -706,7 +706,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">producer</t>
+          <t xml:space="preserve">regulator_england</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -721,12 +721,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Producer</t>
+          <t xml:space="preserve">Environment Agency (England)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cynhyrchydd</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -738,7 +738,7 @@
     <row r="20" ht="51" customHeight="1">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsHeader.en.resx::regulator</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsHeader.en.resx::regulator_northern_ireland</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -748,7 +748,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">regulator</t>
+          <t xml:space="preserve">regulator_northern_ireland</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -763,12 +763,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Regulator</t>
+          <t xml:space="preserve">Environment Agency (Northern Ireland)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rheoleiddiwr</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -780,7 +780,7 @@
     <row r="21" ht="51" customHeight="1">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsHeader.en.resx::regulator_england</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsHeader.en.resx::regulator_scotland</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">regulator_england</t>
+          <t xml:space="preserve">regulator_scotland</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Environment Agency (England)</t>
+          <t xml:space="preserve">Environment Agency (Scotland)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -822,7 +822,7 @@
     <row r="22" ht="51" customHeight="1">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsHeader.en.resx::regulator_northern_ireland</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsHeader.en.resx::regulator_wales</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">regulator_northern_ireland</t>
+          <t xml:space="preserve">regulator_wales</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Environment Agency (Northern Ireland)</t>
+          <t xml:space="preserve">Environment Agency (Wales)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -864,17 +864,17 @@
     <row r="23" ht="51" customHeight="1">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsHeader.en.resx::regulator_scotland</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_numberOfPrns.en.resx::number_of_prns_and_perns_awaiting_acceptance</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsHeader.en.resx</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_numberOfPrns.en.resx</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">regulator_scotland</t>
+          <t xml:space="preserve">number_of_prns_and_perns_awaiting_acceptance</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -889,12 +889,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Environment Agency (Scotland)</t>
+          <t xml:space="preserve">Number of PRNs and PERNs awaiting acceptance</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Nifer y PRNs a'r PERNs sy'n aros i gael eu derbyn</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -906,17 +906,17 @@
     <row r="24" ht="51" customHeight="1">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsHeader.en.resx::regulator_wales</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_numberOfPrns.en.resx::accept_or_reject_prns_and_perns</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsHeader.en.resx</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_numberOfPrns.en.resx</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">regulator_wales</t>
+          <t xml:space="preserve">accept_or_reject_prns_and_perns</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -931,12 +931,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Environment Agency (Wales)</t>
+          <t xml:space="preserve">Accept or reject PRNs and PERNs</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Derbyn neu wrthod PRNs a PERNs</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -948,17 +948,17 @@
     <row r="25" ht="51" customHeight="1">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_numberOfPrns.en.resx::number_of_prns_and_perns_awaiting_acceptance</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::arialabel_aluminium</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_numberOfPrns.en.resx</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">number_of_prns_and_perns_awaiting_acceptance</t>
+          <t xml:space="preserve">arialabel_aluminium</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -973,12 +973,12 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Number of PRNs and PERNs awaiting acceptance</t>
+          <t xml:space="preserve">Aluminium recycling obligation page</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nifer y PRNs a'r PERNs sy'n aros i gael eu derbyn</t>
+          <t xml:space="preserve">Tudalen rhwymedigaethau ailgylchu alwminiwm</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -990,17 +990,17 @@
     <row r="26" ht="51" customHeight="1">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_numberOfPrns.en.resx::accept_or_reject_prns_and_perns</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::aluminium</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_numberOfPrns.en.resx</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">accept_or_reject_prns_and_perns</t>
+          <t xml:space="preserve">aluminium</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1015,12 +1015,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accept or reject PRNs and PERNs</t>
+          <t xml:space="preserve">Aluminium</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Derbyn neu wrthod PRNs a PERNs</t>
+          <t xml:space="preserve">Alwminiwm</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1032,7 +1032,7 @@
     <row r="27" ht="51" customHeight="1">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::arialabel_aluminium</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::arialabel_glass</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">arialabel_aluminium</t>
+          <t xml:space="preserve">arialabel_glass</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1057,12 +1057,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aluminium recycling obligation page</t>
+          <t xml:space="preserve">Glass recycling obligation page</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tudalen rhwymedigaethau ailgylchu alwminiwm</t>
+          <t xml:space="preserve">Tudalen rhwymedigaethau ailgylchu gwydr</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1074,7 +1074,7 @@
     <row r="28" ht="51" customHeight="1">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::aluminium</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::glass</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">aluminium</t>
+          <t xml:space="preserve">glass</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1099,12 +1099,12 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aluminium</t>
+          <t xml:space="preserve">Glass</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alwminiwm</t>
+          <t xml:space="preserve">Gwydr</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1116,7 +1116,7 @@
     <row r="29" ht="51" customHeight="1">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::arialabel_glass</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::glass_recycling_obligation_breakdown</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">arialabel_glass</t>
+          <t xml:space="preserve">glass_recycling_obligation_breakdown</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1141,12 +1141,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Glass recycling obligation page</t>
+          <t xml:space="preserve">Glass recycling obligation breakdown</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tudalen rhwymedigaethau ailgylchu gwydr</t>
+          <t xml:space="preserve">Dadansoddiad o'r rhwymedigaeth ailgylchu gwydr</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1158,7 +1158,7 @@
     <row r="30" ht="51" customHeight="1">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::glass</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::arialabel_glass_remelt</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">glass</t>
+          <t xml:space="preserve">arialabel_glass_remelt</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1183,12 +1183,12 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Glass</t>
+          <t xml:space="preserve">Glass re-melt recycling obligation page</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gwydr</t>
+          <t xml:space="preserve">Tudalen rhwymedigaethau ailgylchu gwydr aildoddi</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1200,7 +1200,7 @@
     <row r="31" ht="51" customHeight="1">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::glass_recycling_obligation_breakdown</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::glass_remelt</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1210,7 +1210,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">glass_recycling_obligation_breakdown</t>
+          <t xml:space="preserve">glass_remelt</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1225,12 +1225,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Glass recycling obligation breakdown</t>
+          <t xml:space="preserve">Glass re-melt</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dadansoddiad o'r rhwymedigaeth ailgylchu gwydr</t>
+          <t xml:space="preserve">Gwydr aildoddi</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1242,7 +1242,7 @@
     <row r="32" ht="51" customHeight="1">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::arialabel_glass_remelt</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::material</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">arialabel_glass_remelt</t>
+          <t xml:space="preserve">material</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1267,12 +1267,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Glass re-melt recycling obligation page</t>
+          <t xml:space="preserve">Material</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tudalen rhwymedigaethau ailgylchu gwydr aildoddi</t>
+          <t xml:space="preserve">Deunydd</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1284,7 +1284,7 @@
     <row r="33" ht="51" customHeight="1">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::glass_remelt</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::met</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">glass_remelt</t>
+          <t xml:space="preserve">met</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1309,12 +1309,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Glass re-melt</t>
+          <t xml:space="preserve">Met</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gwydr aildoddi</t>
+          <t xml:space="preserve">Wedi'i gyflawni</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1326,7 +1326,7 @@
     <row r="34" ht="51" customHeight="1">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::material</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::not_available_yet</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1336,7 +1336,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">material</t>
+          <t xml:space="preserve">not_available_yet</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1351,12 +1351,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Material</t>
+          <t xml:space="preserve">Not available yet</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deunydd</t>
+          <t xml:space="preserve">Heb fod ar gael eto</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1368,7 +1368,7 @@
     <row r="35" ht="51" customHeight="1">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::met</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::not_met</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">met</t>
+          <t xml:space="preserve">not_met</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1393,12 +1393,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Met</t>
+          <t xml:space="preserve">Not met</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wedi'i gyflawni</t>
+          <t xml:space="preserve">Heb ei gyflawni</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1410,7 +1410,7 @@
     <row r="36" ht="51" customHeight="1">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::not_available_yet</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::no_data_yet</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1420,7 +1420,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">not_available_yet</t>
+          <t xml:space="preserve">no_data_yet</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1435,12 +1435,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not available yet</t>
+          <t xml:space="preserve">No data yet</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Heb fod ar gael eto</t>
+          <t xml:space="preserve">Dim data eto</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1452,7 +1452,7 @@
     <row r="37" ht="51" customHeight="1">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::not_met</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::arialabel_paper_board_fibre</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">not_met</t>
+          <t xml:space="preserve">arialabel_paper_board_fibre</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1477,12 +1477,12 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not met</t>
+          <t xml:space="preserve">Paper, board or fibre-based composite material recycling obligation page</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Heb ei gyflawni</t>
+          <t xml:space="preserve">Tudalen rhwymedigaethau ailgylchu papur, bwrdd neu ddeunydd cyfansawdd sy'n seiliedig ar ffeibrau</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1494,7 +1494,7 @@
     <row r="38" ht="51" customHeight="1">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::no_data_yet</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::paper_board_fibre</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">no_data_yet</t>
+          <t xml:space="preserve">paper_board_fibre</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1519,12 +1519,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t xml:space="preserve">No data yet</t>
+          <t xml:space="preserve">Paper, board or fibre-based composite material</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dim data eto</t>
+          <t xml:space="preserve">Papur, bwrdd neu ddeunydd cyfansawdd sy'n seiliedig ar ffeibrau</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -1536,7 +1536,7 @@
     <row r="39" ht="51" customHeight="1">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::arialabel_paper_board_fibre</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::arialabel_plastic</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1546,7 +1546,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">arialabel_paper_board_fibre</t>
+          <t xml:space="preserve">arialabel_plastic</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1561,12 +1561,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paper, board or fibre-based composite material recycling obligation page</t>
+          <t xml:space="preserve">Plastic recycling obligation page</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tudalen rhwymedigaethau ailgylchu papur, bwrdd neu ddeunydd cyfansawdd sy'n seiliedig ar ffeibrau</t>
+          <t xml:space="preserve">Tudalen rhwymedigaethau ailgylchu plastigau</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -1578,7 +1578,7 @@
     <row r="40" ht="51" customHeight="1">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::paper_board_fibre</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::plastic</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1588,7 +1588,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">paper_board_fibre</t>
+          <t xml:space="preserve">plastic</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1603,12 +1603,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paper, board or fibre-based composite material</t>
+          <t xml:space="preserve">Plastic</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Papur, bwrdd neu ddeunydd cyfansawdd sy'n seiliedig ar ffeibrau</t>
+          <t xml:space="preserve">Plastig</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -1620,7 +1620,7 @@
     <row r="41" ht="51" customHeight="1">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::arialabel_plastic</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::recycling_obligations_to_meet</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">arialabel_plastic</t>
+          <t xml:space="preserve">recycling_obligations_to_meet</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1645,12 +1645,12 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plastic recycling obligation page</t>
+          <t xml:space="preserve">Recycling obligations to meet</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tudalen rhwymedigaethau ailgylchu plastigau</t>
+          <t xml:space="preserve">Rhwymedigaethau ailgylchu i'w cyflawni</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -1662,7 +1662,7 @@
     <row r="42" ht="51" customHeight="1">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::plastic</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::arialabel_remaining_glass</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1672,7 +1672,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">plastic</t>
+          <t xml:space="preserve">arialabel_remaining_glass</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1687,12 +1687,12 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plastic</t>
+          <t xml:space="preserve">Remaining glass recycling obligation page</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plastig</t>
+          <t xml:space="preserve">Tudalen rhwymedigaethau ailgylchu gweddill y gwydr</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -1704,7 +1704,7 @@
     <row r="43" ht="51" customHeight="1">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::recycling_obligations_to_meet</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::remaining_glass</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">recycling_obligations_to_meet</t>
+          <t xml:space="preserve">remaining_glass</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1729,12 +1729,12 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recycling obligations to meet</t>
+          <t xml:space="preserve">Remaining glass</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rhwymedigaethau ailgylchu i'w cyflawni</t>
+          <t xml:space="preserve">Gweddill y gwydr</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -1746,7 +1746,7 @@
     <row r="44" ht="51" customHeight="1">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::arialabel_remaining_glass</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::status</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1756,7 +1756,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">arialabel_remaining_glass</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1771,12 +1771,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Remaining glass recycling obligation page</t>
+          <t xml:space="preserve">Status</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tudalen rhwymedigaethau ailgylchu gweddill y gwydr</t>
+          <t xml:space="preserve">Statws</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -1788,7 +1788,7 @@
     <row r="45" ht="51" customHeight="1">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::remaining_glass</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::arialabel_steel</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">remaining_glass</t>
+          <t xml:space="preserve">arialabel_steel</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1813,12 +1813,12 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Remaining glass</t>
+          <t xml:space="preserve">Steel recycling obligation page</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gweddill y gwydr</t>
+          <t xml:space="preserve">Tudalen rhwymedigaethau ailgylchu dur</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -1830,7 +1830,7 @@
     <row r="46" ht="51" customHeight="1">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::status</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::steel</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">steel</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1855,12 +1855,12 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Status</t>
+          <t xml:space="preserve">Steel</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Statws</t>
+          <t xml:space="preserve">Dur</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -1872,7 +1872,7 @@
     <row r="47" ht="51" customHeight="1">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::arialabel_steel</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::tonnage_accepted</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1882,7 +1882,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">arialabel_steel</t>
+          <t xml:space="preserve">tonnage_accepted</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1897,12 +1897,12 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Steel recycling obligation page</t>
+          <t xml:space="preserve">Tonnage accepted</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tudalen rhwymedigaethau ailgylchu dur</t>
+          <t xml:space="preserve">Tunelli wedi'u derbyn</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -1914,7 +1914,7 @@
     <row r="48" ht="51" customHeight="1">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::steel</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::tonnage_awaiting_acceptance</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">steel</t>
+          <t xml:space="preserve">tonnage_awaiting_acceptance</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1939,12 +1939,12 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Steel</t>
+          <t xml:space="preserve">Tonnage awaiting acceptance</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dur</t>
+          <t xml:space="preserve">Tunelli yn aros i gael eu derbyn</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -1956,7 +1956,7 @@
     <row r="49" ht="51" customHeight="1">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::tonnage_accepted</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::tonnage_outstanding</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">tonnage_accepted</t>
+          <t xml:space="preserve">tonnage_outstanding</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1981,12 +1981,12 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tonnage accepted</t>
+          <t xml:space="preserve">Tonnage outstanding</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tunelli wedi'u derbyn</t>
+          <t xml:space="preserve">Tunelli sy'n weddill</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -1998,7 +1998,7 @@
     <row r="50" ht="51" customHeight="1">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::tonnage_awaiting_acceptance</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::totals</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2008,7 +2008,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">tonnage_awaiting_acceptance</t>
+          <t xml:space="preserve">totals</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2023,12 +2023,12 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tonnage awaiting acceptance</t>
+          <t xml:space="preserve">Totals</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tunelli yn aros i gael eu derbyn</t>
+          <t xml:space="preserve">Cyfansymiau</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2040,7 +2040,7 @@
     <row r="51" ht="51" customHeight="1">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::tonnage_outstanding</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::arialabel_wood</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">tonnage_outstanding</t>
+          <t xml:space="preserve">arialabel_wood</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2065,12 +2065,12 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tonnage outstanding</t>
+          <t xml:space="preserve">Wood recycling obligation page</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tunelli sy'n weddill</t>
+          <t xml:space="preserve">Tudalen rhwymedigaethau ailgylchu pren</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2082,7 +2082,7 @@
     <row r="52" ht="51" customHeight="1">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::totals</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::wood</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2092,7 +2092,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">totals</t>
+          <t xml:space="preserve">wood</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2107,12 +2107,12 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Totals</t>
+          <t xml:space="preserve">Wood</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cyfansymiau</t>
+          <t xml:space="preserve">Pren</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2124,7 +2124,7 @@
     <row r="53" ht="51" customHeight="1">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::arialabel_wood</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::your_recycling_obligations_progress</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2134,7 +2134,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">arialabel_wood</t>
+          <t xml:space="preserve">your_recycling_obligations_progress</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2149,12 +2149,12 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wood recycling obligation page</t>
+          <t xml:space="preserve">Your recycling obligations progress</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tudalen rhwymedigaethau ailgylchu pren</t>
+          <t xml:space="preserve">Cynnydd eich rhwymedigaethau ailgylchu</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -2166,17 +2166,17 @@
     <row r="54" ht="51" customHeight="1">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::wood</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_heading</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t xml:space="preserve">wood</t>
+          <t xml:space="preserve">obligations_details_summary_heading</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2191,12 +2191,12 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wood</t>
+          <t xml:space="preserve">Why does the recycling obligations table already have tonnage awaiting acceptance?</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pren</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2208,17 +2208,17 @@
     <row r="55" ht="51" customHeight="1">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx::your_recycling_obligations_progress</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_intro</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_prnMaterialTable.en.resx</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">your_recycling_obligations_progress</t>
+          <t xml:space="preserve">obligations_details_summary_content_intro</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2233,12 +2233,12 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Your recycling obligations progress</t>
+          <t xml:space="preserve">Tonnage awaiting acceptance is for PRNs or PERNs that have been issued to you but have not yet been accepted.</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cynnydd eich rhwymedigaethau ailgylchu</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -2250,7 +2250,7 @@
     <row r="56" ht="51" customHeight="1">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_heading</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_before_list_1</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve">obligations_details_summary_heading</t>
+          <t xml:space="preserve">obligations_details_summary_content_before_list_1</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Why does the recycling obligations table already have tonnage awaiting acceptance?</t>
+          <t xml:space="preserve">You have been issued at least one December waste PRN or PERN.</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2292,7 +2292,7 @@
     <row r="57" ht="51" customHeight="1">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_intro</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_before_list_2</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2302,7 +2302,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">obligations_details_summary_content_intro</t>
+          <t xml:space="preserve">obligations_details_summary_content_before_list_2</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2317,7 +2317,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tonnage awaiting acceptance is for PRNs or PERNs that have been issued to you but have not yet been accepted.</t>
+          <t xml:space="preserve">These:</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2334,7 +2334,7 @@
     <row r="58" ht="51" customHeight="1">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_before_list_1</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_bullet_1</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">obligations_details_summary_content_before_list_1</t>
+          <t xml:space="preserve">obligations_details_summary_content_bullet_1</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t xml:space="preserve">You have been issued at least one December waste PRN or PERN.</t>
+          <t xml:space="preserve">are for packaging waste received for recycling at UK or overseas reprocessing sites in December</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2376,7 +2376,7 @@
     <row r="59" ht="51" customHeight="1">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_before_list_2</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_bullet_2</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve">obligations_details_summary_content_before_list_2</t>
+          <t xml:space="preserve">obligations_details_summary_content_bullet_2</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2401,7 +2401,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t xml:space="preserve">These:</t>
+          <t xml:space="preserve">can be accepted towards either your {0} or {1} recycling obligations</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2418,7 +2418,7 @@
     <row r="60" ht="51" customHeight="1">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_bullet_1</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_bullet_3</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2428,7 +2428,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">obligations_details_summary_content_bullet_1</t>
+          <t xml:space="preserve">obligations_details_summary_content_bullet_3</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t xml:space="preserve">are for packaging waste received for recycling at UK or overseas reprocessing sites in December</t>
+          <t xml:space="preserve">have a blue tag to show which years you can accept them towards</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2460,7 +2460,7 @@
     <row r="61" ht="51" customHeight="1">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_bullet_2</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_after_list</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2470,7 +2470,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">obligations_details_summary_content_bullet_2</t>
+          <t xml:space="preserve">obligations_details_summary_content_after_list</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2485,7 +2485,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t xml:space="preserve">can be accepted towards either your {0} or {1} recycling obligations</t>
+          <t xml:space="preserve">A December waste PRN or PERN will appear under ‘Tonnage awaiting acceptance’ for both {0} and {1} until you accept it towards a specific year’s recycling obligations.</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2502,7 +2502,7 @@
     <row r="62" ht="51" customHeight="1">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_bullet_3</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_end</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2512,7 +2512,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">obligations_details_summary_content_bullet_3</t>
+          <t xml:space="preserve">obligations_details_summary_content_end</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t xml:space="preserve">have a blue tag to show which years you can accept them towards</t>
+          <t xml:space="preserve">Once you accept the PRN or PERN towards a specific year, it is assigned to that year only and the blue tag is removed.</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2544,17 +2544,17 @@
     <row r="63" ht="51" customHeight="1">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_after_list</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_meetingObligations.en.resx::meeting_obligations_list_1_prefix</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_meetingObligations.en.resx</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">obligations_details_summary_content_after_list</t>
+          <t xml:space="preserve">meeting_obligations_list_1_prefix</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2569,7 +2569,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t xml:space="preserve">A December waste PRN or PERN will appear under ‘Tonnage awaiting acceptance’ for both {0} and {1} until you accept it towards a specific year’s recycling obligations.</t>
+          <t xml:space="preserve">Your {0} recycling obligations have not been calculated yet. They will be calculated after:</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -2586,17 +2586,17 @@
     <row r="64" ht="51" customHeight="1">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx::obligations_details_summary_content_end</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_meetingObligations.en.resx::meeting_obligations_list_1_bullet_1</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_obligationsDetailsSummary.en.resx</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_meetingObligations.en.resx</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t xml:space="preserve">obligations_details_summary_content_end</t>
+          <t xml:space="preserve">meeting_obligations_list_1_bullet_1</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Once you accept the PRN or PERN towards a specific year, it is assigned to that year only and the blue tag is removed.</t>
+          <t xml:space="preserve">you submit your packaging data for {0}</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -2625,8 +2625,218 @@
         </is>
       </c>
     </row>
+    <row r="65" ht="51" customHeight="1">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_meetingObligations.en.resx::meeting_obligations_list_1_bullet_2</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_meetingObligations.en.resx</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">meeting_obligations_list_1_bullet_2</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prns-obligations-home-no-obligations</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/manage-your-recycling-obligations</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">your environmental regulator accepts your H1 and H2 packaging data submissions</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=1915-112595</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="51" customHeight="1">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_meetingObligations.en.resx::meeting_obligations_list_2_prefix</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_meetingObligations.en.resx</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">meeting_obligations_list_2_prefix</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prns-obligations-home-no-obligations</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/manage-your-recycling-obligations</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Until then, you can:</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=1915-112595</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="51" customHeight="1">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_meetingObligations.en.resx::meeting_obligations_list_2_bullet_1</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_meetingObligations.en.resx</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">meeting_obligations_list_2_bullet_1</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prns-obligations-home-no-obligations</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/manage-your-recycling-obligations</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">acquire packaging waste recycling notes (PRNs) and packaging waste export recycling notes (PERNs)</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=1915-112595</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="51" customHeight="1">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_meetingObligations.en.resx::meeting_obligations_list_2_bullet_2</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_meetingObligations.en.resx</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">meeting_obligations_list_2_bullet_2</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prns-obligations-home-no-obligations</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/manage-your-recycling-obligations</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accept your PRNs and PERNs towards your recycling obligations</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=1915-112595</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="51" customHeight="1">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_meetingObligations.en.resx::meeting_obligations_table_below_statement</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_meetingObligations.en.resx</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">meeting_obligations_table_below_statement</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prns-obligations-home-no-obligations</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/manage-your-recycling-obligations</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You will see data for PRNs and PERNs you have acquired in the table below. But you will only see progress against your actual recycling obligations once they have been calculated.</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=1915-112595</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:H64"/>
+  <autoFilter ref="A5:H69"/>
   <mergeCells count="3">
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="F2:H2"/>

</xml_diff>